<commit_message>
Complete company-admin invite flow and refresh trackers
</commit_message>
<xml_diff>
--- a/docs/done.xlsx
+++ b/docs/done.xlsx
@@ -1,9 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <workbookViews>
-    <workbookView/>
-  </workbookViews>
   <sheets>
     <sheet name="Done" sheetId="1" r:id="rId1"/>
   </sheets>
@@ -15,7 +12,7 @@
   <fonts count="1">
     <font>
       <sz val="11"/>
-      <name val="Arial"/>
+      <name val="Aptos"/>
     </font>
   </fonts>
   <fills count="2">
@@ -49,7 +46,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">

</xml_diff>